<commit_message>
previous commit's message should be for this...
</commit_message>
<xml_diff>
--- a/model_modifications/inputs/reactions_additions_v9.xlsx
+++ b/model_modifications/inputs/reactions_additions_v9.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\inapa\PycharmProjects\metabolic_modeling\model_modifications\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B89E3174-FFAB-4C4E-A11C-DEFA9B84696A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6A39E3-0B68-40AB-B583-D9239E155E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2565" yWindow="-11835" windowWidth="20685" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-45" yWindow="-15870" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rxns" sheetId="1" r:id="rId1"/>
@@ -1637,9 +1637,6 @@
     <t>AKR1D1 </t>
   </si>
   <si>
-    <t>SULT1E1 or SULT1A1 or SULT1A3</t>
-  </si>
-  <si>
     <t>AKR1D1</t>
   </si>
   <si>
@@ -1764,6 +1761,9 @@
   </si>
   <si>
     <t>MAR90038</t>
+  </si>
+  <si>
+    <t>SULT1E1 or ENSG00000196502 or SULT1A3</t>
   </si>
 </sst>
 </file>
@@ -5721,22 +5721,22 @@
         <v>12</v>
       </c>
       <c r="G157" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H157" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I157" t="s">
+        <v>557</v>
+      </c>
+      <c r="J157" t="s">
         <v>558</v>
-      </c>
-      <c r="J157" t="s">
-        <v>559</v>
       </c>
       <c r="K157" t="s">
         <v>529</v>
       </c>
       <c r="L157" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.3">
@@ -5744,22 +5744,22 @@
         <v>12</v>
       </c>
       <c r="G158" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="H158" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="I158" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J158" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="K158" t="s">
         <v>530</v>
       </c>
       <c r="L158" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.3">
@@ -5767,22 +5767,22 @@
         <v>12</v>
       </c>
       <c r="G159" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="H159" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="I159" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J159" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="K159" t="s">
         <v>531</v>
       </c>
       <c r="L159" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.3">
@@ -5790,22 +5790,22 @@
         <v>12</v>
       </c>
       <c r="G160" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="H160" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="I160" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J160" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="K160" t="s">
         <v>532</v>
       </c>
       <c r="L160" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.3">
@@ -5813,22 +5813,22 @@
         <v>12</v>
       </c>
       <c r="G161" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="H161" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I161" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J161" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="K161" t="s">
         <v>529</v>
       </c>
       <c r="L161" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.3">
@@ -5836,22 +5836,22 @@
         <v>12</v>
       </c>
       <c r="G162" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="H162" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="I162" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J162" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="K162" t="s">
         <v>530</v>
       </c>
       <c r="L162" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.3">
@@ -5859,22 +5859,22 @@
         <v>12</v>
       </c>
       <c r="G163" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H163" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="I163" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J163" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="K163" t="s">
         <v>531</v>
       </c>
       <c r="L163" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.3">
@@ -5882,22 +5882,22 @@
         <v>12</v>
       </c>
       <c r="G164" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="H164" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="I164" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J164" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="K164" t="s">
-        <v>533</v>
+        <v>575</v>
       </c>
       <c r="L164" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.3">
@@ -5905,22 +5905,22 @@
         <v>12</v>
       </c>
       <c r="G165" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H165" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="I165" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J165" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="K165" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L165" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.3">
@@ -5928,22 +5928,22 @@
         <v>12</v>
       </c>
       <c r="G166" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H166" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="I166" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J166" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="K166" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L166" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="167" spans="1:12" x14ac:dyDescent="0.3">
@@ -5951,22 +5951,22 @@
         <v>12</v>
       </c>
       <c r="G167" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="H167" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="I167" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J167" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="K167" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L167" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="168" spans="1:12" x14ac:dyDescent="0.3">
@@ -5974,22 +5974,22 @@
         <v>12</v>
       </c>
       <c r="G168" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="H168" t="s">
+        <v>556</v>
+      </c>
+      <c r="I168" t="s">
         <v>557</v>
       </c>
-      <c r="I168" t="s">
-        <v>558</v>
-      </c>
       <c r="J168" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="K168" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="L168" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="169" spans="1:12" x14ac:dyDescent="0.3">
@@ -5997,42 +5997,42 @@
         <v>12</v>
       </c>
       <c r="G169" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="H169" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="I169" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J169" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="K169" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L169" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="170" spans="1:12" x14ac:dyDescent="0.3">
       <c r="G170" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="H170" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="I170" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J170" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="K170" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L170" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>